<commit_message>
HE missing acc finished
</commit_message>
<xml_diff>
--- a/data/hex_xlsx/AFAGR.HE.xlsx
+++ b/data/hex_xlsx/AFAGR.HE.xlsx
@@ -1901,7 +1901,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1979,6 +1979,12 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="6" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -20490,7 +20496,9 @@
       <c r="H100" s="17">
         <v>325.35</v>
       </c>
-      <c r="I100" s="20"/>
+      <c r="I100" s="30">
+        <v>320.0</v>
+      </c>
       <c r="J100" s="18">
         <v>18.66</v>
       </c>
@@ -20499,8 +20507,12 @@
       </c>
       <c r="L100" s="20"/>
       <c r="M100" s="20"/>
-      <c r="N100" s="20"/>
-      <c r="O100" s="20"/>
+      <c r="N100" s="18">
+        <v>11.36</v>
+      </c>
+      <c r="O100" s="18">
+        <v>19.96</v>
+      </c>
       <c r="P100" s="18">
         <v>8.3</v>
       </c>
@@ -20516,10 +20528,18 @@
       <c r="T100" s="17">
         <v>124.74</v>
       </c>
-      <c r="U100" s="20"/>
-      <c r="V100" s="20"/>
-      <c r="W100" s="20"/>
-      <c r="X100" s="20"/>
+      <c r="U100" s="31">
+        <v>80.0</v>
+      </c>
+      <c r="V100" s="18">
+        <v>24.1</v>
+      </c>
+      <c r="W100" s="18">
+        <v>27.85</v>
+      </c>
+      <c r="X100" s="18">
+        <v>20.75</v>
+      </c>
       <c r="Y100" s="20"/>
       <c r="Z100" s="20"/>
       <c r="AA100" s="20"/>
@@ -29526,10 +29546,10 @@
       <c r="X11" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="Y11" s="30" t="s">
+      <c r="Y11" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="Z11" s="31"/>
+      <c r="Z11" s="33"/>
       <c r="AA11" s="7" t="s">
         <v>42</v>
       </c>
@@ -38121,83 +38141,83 @@
       <c r="A31" s="16" t="s">
         <v>536</v>
       </c>
-      <c r="B31" s="32">
+      <c r="B31" s="34">
         <v>-15.85</v>
       </c>
-      <c r="C31" s="33">
+      <c r="C31" s="35">
         <v>6.12</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D31" s="35">
         <v>32.46</v>
       </c>
-      <c r="E31" s="33">
+      <c r="E31" s="35">
         <v>24.1</v>
       </c>
-      <c r="F31" s="33">
+      <c r="F31" s="35">
         <v>10.79</v>
       </c>
-      <c r="G31" s="32">
+      <c r="G31" s="34">
         <v>-3.12</v>
       </c>
-      <c r="H31" s="32">
+      <c r="H31" s="34">
         <v>-2.35</v>
       </c>
-      <c r="I31" s="32">
+      <c r="I31" s="34">
         <v>-3.11</v>
       </c>
-      <c r="J31" s="33">
+      <c r="J31" s="35">
         <v>2.73</v>
       </c>
-      <c r="K31" s="33">
+      <c r="K31" s="35">
         <v>4.6</v>
       </c>
-      <c r="L31" s="32">
+      <c r="L31" s="34">
         <v>-10.26</v>
       </c>
-      <c r="M31" s="33">
+      <c r="M31" s="35">
         <v>4.29</v>
       </c>
-      <c r="N31" s="33">
+      <c r="N31" s="35">
         <v>2.12</v>
       </c>
-      <c r="O31" s="32">
+      <c r="O31" s="34">
         <v>-6.88</v>
       </c>
-      <c r="P31" s="32">
+      <c r="P31" s="34">
         <v>-4.24</v>
       </c>
-      <c r="Q31" s="32">
+      <c r="Q31" s="34">
         <v>-1.78</v>
       </c>
-      <c r="R31" s="32">
+      <c r="R31" s="34">
         <v>-7.67</v>
       </c>
-      <c r="S31" s="33">
+      <c r="S31" s="35">
         <v>0.54</v>
       </c>
-      <c r="T31" s="33">
+      <c r="T31" s="35">
         <v>2.69</v>
       </c>
-      <c r="U31" s="32">
+      <c r="U31" s="34">
         <v>-3992.48</v>
       </c>
-      <c r="V31" s="33">
+      <c r="V31" s="35">
         <v>16.33</v>
       </c>
-      <c r="W31" s="32">
+      <c r="W31" s="34">
         <v>-173.88</v>
       </c>
-      <c r="X31" s="33"/>
-      <c r="Y31" s="32">
+      <c r="X31" s="35"/>
+      <c r="Y31" s="34">
         <v>-104.14</v>
       </c>
-      <c r="Z31" s="32">
+      <c r="Z31" s="34">
         <v>-1.11</v>
       </c>
-      <c r="AA31" s="33">
+      <c r="AA31" s="35">
         <v>58.04</v>
       </c>
-      <c r="AB31" s="33">
+      <c r="AB31" s="35">
         <v>8.04</v>
       </c>
     </row>
@@ -38205,69 +38225,69 @@
       <c r="A32" s="16" t="s">
         <v>537</v>
       </c>
-      <c r="B32" s="33">
+      <c r="B32" s="35">
         <v>10.67</v>
       </c>
-      <c r="C32" s="33">
+      <c r="C32" s="35">
         <v>10.94</v>
       </c>
-      <c r="D32" s="33">
+      <c r="D32" s="35">
         <v>7.02</v>
       </c>
-      <c r="E32" s="32">
+      <c r="E32" s="34">
         <v>-0.11</v>
       </c>
-      <c r="F32" s="32">
+      <c r="F32" s="34">
         <v>-0.46</v>
       </c>
-      <c r="G32" s="32">
+      <c r="G32" s="34">
         <v>-0.62</v>
       </c>
-      <c r="H32" s="32">
+      <c r="H32" s="34">
         <v>-1.18</v>
       </c>
-      <c r="I32" s="32">
+      <c r="I32" s="34">
         <v>-0.21</v>
       </c>
-      <c r="J32" s="33">
+      <c r="J32" s="35">
         <v>1.34</v>
       </c>
-      <c r="K32" s="32">
+      <c r="K32" s="34">
         <v>-2.19</v>
       </c>
-      <c r="L32" s="32">
+      <c r="L32" s="34">
         <v>-3.88</v>
       </c>
-      <c r="M32" s="32">
+      <c r="M32" s="34">
         <v>-2.7</v>
       </c>
-      <c r="N32" s="32">
+      <c r="N32" s="34">
         <v>-3.94</v>
       </c>
-      <c r="O32" s="32">
+      <c r="O32" s="34">
         <v>-2.84</v>
       </c>
-      <c r="P32" s="32">
+      <c r="P32" s="34">
         <v>-1.7</v>
       </c>
-      <c r="Q32" s="32">
+      <c r="Q32" s="34">
         <v>-315.57</v>
       </c>
-      <c r="R32" s="32">
+      <c r="R32" s="34">
         <v>-405.29</v>
       </c>
-      <c r="S32" s="32">
+      <c r="S32" s="34">
         <v>-466.83</v>
       </c>
-      <c r="T32" s="33"/>
-      <c r="U32" s="33"/>
-      <c r="V32" s="33"/>
-      <c r="W32" s="33"/>
-      <c r="X32" s="33"/>
-      <c r="Y32" s="33"/>
-      <c r="Z32" s="33"/>
-      <c r="AA32" s="33"/>
-      <c r="AB32" s="33"/>
+      <c r="T32" s="35"/>
+      <c r="U32" s="35"/>
+      <c r="V32" s="35"/>
+      <c r="W32" s="35"/>
+      <c r="X32" s="35"/>
+      <c r="Y32" s="35"/>
+      <c r="Z32" s="35"/>
+      <c r="AA32" s="35"/>
+      <c r="AB32" s="35"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="14" t="s">
@@ -38305,81 +38325,81 @@
       <c r="A34" s="16" t="s">
         <v>539</v>
       </c>
-      <c r="B34" s="33">
+      <c r="B34" s="35">
         <v>0.0</v>
       </c>
-      <c r="C34" s="33">
+      <c r="C34" s="35">
         <v>0.0</v>
       </c>
-      <c r="D34" s="33">
+      <c r="D34" s="35">
         <v>0.0</v>
       </c>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33">
+      <c r="E34" s="35"/>
+      <c r="F34" s="35">
         <v>0.0</v>
       </c>
-      <c r="G34" s="33">
+      <c r="G34" s="35">
         <v>0.0</v>
       </c>
-      <c r="H34" s="33">
+      <c r="H34" s="35">
         <v>0.0</v>
       </c>
-      <c r="I34" s="33">
+      <c r="I34" s="35">
         <v>2.37</v>
       </c>
-      <c r="J34" s="33">
+      <c r="J34" s="35">
         <v>2.58</v>
       </c>
-      <c r="K34" s="33">
+      <c r="K34" s="35">
         <v>4.98</v>
       </c>
-      <c r="L34" s="33">
+      <c r="L34" s="35">
         <v>6.29</v>
       </c>
-      <c r="M34" s="33">
+      <c r="M34" s="35">
         <v>0.0</v>
       </c>
-      <c r="N34" s="33">
+      <c r="N34" s="35">
         <v>0.0</v>
       </c>
-      <c r="O34" s="33">
+      <c r="O34" s="35">
         <v>0.0</v>
       </c>
-      <c r="P34" s="33">
+      <c r="P34" s="35">
         <v>0.0</v>
       </c>
-      <c r="Q34" s="33">
+      <c r="Q34" s="35">
         <v>0.0</v>
       </c>
-      <c r="R34" s="33">
+      <c r="R34" s="35">
         <v>2.93</v>
       </c>
-      <c r="S34" s="33">
+      <c r="S34" s="35">
         <v>0.9</v>
       </c>
-      <c r="T34" s="33">
+      <c r="T34" s="35">
         <v>2.11</v>
       </c>
-      <c r="U34" s="33">
+      <c r="U34" s="35">
         <v>0.0</v>
       </c>
-      <c r="V34" s="33">
+      <c r="V34" s="35">
         <v>0.0</v>
       </c>
-      <c r="W34" s="33">
+      <c r="W34" s="35">
         <v>0.0</v>
       </c>
-      <c r="X34" s="33"/>
-      <c r="Y34" s="33">
+      <c r="X34" s="35"/>
+      <c r="Y34" s="35">
         <v>0.0</v>
       </c>
-      <c r="Z34" s="33">
+      <c r="Z34" s="35">
         <v>0.0</v>
       </c>
-      <c r="AA34" s="33">
+      <c r="AA34" s="35">
         <v>0.0</v>
       </c>
-      <c r="AB34" s="33">
+      <c r="AB34" s="35">
         <v>7.87</v>
       </c>
     </row>
@@ -38387,147 +38407,147 @@
       <c r="A35" s="16" t="s">
         <v>540</v>
       </c>
-      <c r="B35" s="33">
+      <c r="B35" s="35">
         <v>0.0</v>
       </c>
-      <c r="C35" s="33">
+      <c r="C35" s="35">
         <v>0.0</v>
       </c>
-      <c r="D35" s="33">
+      <c r="D35" s="35">
         <v>0.0</v>
       </c>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33">
+      <c r="E35" s="35"/>
+      <c r="F35" s="35">
         <v>1.29</v>
       </c>
-      <c r="G35" s="33">
+      <c r="G35" s="35">
         <v>1.83</v>
       </c>
-      <c r="H35" s="33">
+      <c r="H35" s="35">
         <v>2.61</v>
       </c>
-      <c r="I35" s="33">
+      <c r="I35" s="35">
         <v>3.01</v>
       </c>
-      <c r="J35" s="33">
+      <c r="J35" s="35">
         <v>2.65</v>
       </c>
-      <c r="K35" s="33">
+      <c r="K35" s="35">
         <v>1.68</v>
       </c>
-      <c r="L35" s="33">
+      <c r="L35" s="35">
         <v>0.54</v>
       </c>
-      <c r="M35" s="33">
+      <c r="M35" s="35">
         <v>0.0</v>
       </c>
-      <c r="N35" s="33">
+      <c r="N35" s="35">
         <v>0.52</v>
       </c>
-      <c r="O35" s="33">
+      <c r="O35" s="35">
         <v>0.66</v>
       </c>
-      <c r="P35" s="33">
+      <c r="P35" s="35">
         <v>0.92</v>
       </c>
-      <c r="Q35" s="33">
+      <c r="Q35" s="35">
         <v>1.05</v>
       </c>
-      <c r="R35" s="33">
+      <c r="R35" s="35">
         <v>1.36</v>
       </c>
-      <c r="S35" s="33">
+      <c r="S35" s="35">
         <v>0.91</v>
       </c>
-      <c r="T35" s="33"/>
-      <c r="U35" s="33"/>
-      <c r="V35" s="33"/>
-      <c r="W35" s="33"/>
-      <c r="X35" s="33"/>
-      <c r="Y35" s="33"/>
-      <c r="Z35" s="33"/>
-      <c r="AA35" s="33"/>
-      <c r="AB35" s="33"/>
+      <c r="T35" s="35"/>
+      <c r="U35" s="35"/>
+      <c r="V35" s="35"/>
+      <c r="W35" s="35"/>
+      <c r="X35" s="35"/>
+      <c r="Y35" s="35"/>
+      <c r="Z35" s="35"/>
+      <c r="AA35" s="35"/>
+      <c r="AB35" s="35"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="16" t="s">
         <v>541</v>
       </c>
-      <c r="B36" s="33">
+      <c r="B36" s="35">
         <v>0.0</v>
       </c>
-      <c r="C36" s="33">
+      <c r="C36" s="35">
         <v>0.0</v>
       </c>
-      <c r="D36" s="33">
+      <c r="D36" s="35">
         <v>0.0</v>
       </c>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33">
+      <c r="E36" s="35"/>
+      <c r="F36" s="35">
         <v>0.0</v>
       </c>
-      <c r="G36" s="33">
+      <c r="G36" s="35">
         <v>0.0</v>
       </c>
-      <c r="H36" s="33">
+      <c r="H36" s="35">
         <v>0.0</v>
       </c>
-      <c r="I36" s="33">
+      <c r="I36" s="35">
         <v>2.37</v>
       </c>
-      <c r="J36" s="33">
+      <c r="J36" s="35">
         <v>2.58</v>
       </c>
-      <c r="K36" s="33">
+      <c r="K36" s="35">
         <v>4.98</v>
       </c>
-      <c r="L36" s="33">
+      <c r="L36" s="35">
         <v>6.29</v>
       </c>
-      <c r="M36" s="33">
+      <c r="M36" s="35">
         <v>0.0</v>
       </c>
-      <c r="N36" s="33">
+      <c r="N36" s="35">
         <v>0.0</v>
       </c>
-      <c r="O36" s="33">
+      <c r="O36" s="35">
         <v>0.0</v>
       </c>
-      <c r="P36" s="33">
+      <c r="P36" s="35">
         <v>0.0</v>
       </c>
-      <c r="Q36" s="33">
+      <c r="Q36" s="35">
         <v>0.0</v>
       </c>
-      <c r="R36" s="33">
+      <c r="R36" s="35">
         <v>3.65</v>
       </c>
-      <c r="S36" s="33">
+      <c r="S36" s="35">
         <v>1.11</v>
       </c>
-      <c r="T36" s="33">
+      <c r="T36" s="35">
         <v>2.62</v>
       </c>
-      <c r="U36" s="33">
+      <c r="U36" s="35">
         <v>0.0</v>
       </c>
-      <c r="V36" s="33">
+      <c r="V36" s="35">
         <v>0.0</v>
       </c>
-      <c r="W36" s="33">
+      <c r="W36" s="35">
         <v>0.0</v>
       </c>
-      <c r="X36" s="33"/>
-      <c r="Y36" s="33">
+      <c r="X36" s="35"/>
+      <c r="Y36" s="35">
         <v>0.0</v>
       </c>
-      <c r="Z36" s="33">
+      <c r="Z36" s="35">
         <v>0.0</v>
       </c>
-      <c r="AA36" s="33">
+      <c r="AA36" s="35">
         <v>0.0</v>
       </c>
-      <c r="AB36" s="33">
+      <c r="AB36" s="35">
         <v>7.87</v>
       </c>
     </row>
@@ -38535,67 +38555,67 @@
       <c r="A37" s="16" t="s">
         <v>542</v>
       </c>
-      <c r="B37" s="33">
+      <c r="B37" s="35">
         <v>0.0</v>
       </c>
-      <c r="C37" s="33">
+      <c r="C37" s="35">
         <v>0.0</v>
       </c>
-      <c r="D37" s="33">
+      <c r="D37" s="35">
         <v>0.0</v>
       </c>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33">
+      <c r="E37" s="35"/>
+      <c r="F37" s="35">
         <v>1.29</v>
       </c>
-      <c r="G37" s="33">
+      <c r="G37" s="35">
         <v>1.83</v>
       </c>
-      <c r="H37" s="33">
+      <c r="H37" s="35">
         <v>2.61</v>
       </c>
-      <c r="I37" s="33">
+      <c r="I37" s="35">
         <v>3.01</v>
       </c>
-      <c r="J37" s="33">
+      <c r="J37" s="35">
         <v>2.65</v>
       </c>
-      <c r="K37" s="33">
+      <c r="K37" s="35">
         <v>1.68</v>
       </c>
-      <c r="L37" s="33">
+      <c r="L37" s="35">
         <v>0.54</v>
       </c>
-      <c r="M37" s="33">
+      <c r="M37" s="35">
         <v>0.0</v>
       </c>
-      <c r="N37" s="33">
+      <c r="N37" s="35">
         <v>0.64</v>
       </c>
-      <c r="O37" s="33">
+      <c r="O37" s="35">
         <v>0.83</v>
       </c>
-      <c r="P37" s="33">
+      <c r="P37" s="35">
         <v>1.15</v>
       </c>
-      <c r="Q37" s="33">
+      <c r="Q37" s="35">
         <v>1.31</v>
       </c>
-      <c r="R37" s="33">
+      <c r="R37" s="35">
         <v>1.69</v>
       </c>
-      <c r="S37" s="33">
+      <c r="S37" s="35">
         <v>1.13</v>
       </c>
-      <c r="T37" s="33"/>
-      <c r="U37" s="33"/>
-      <c r="V37" s="33"/>
-      <c r="W37" s="33"/>
-      <c r="X37" s="33"/>
-      <c r="Y37" s="33"/>
-      <c r="Z37" s="33"/>
-      <c r="AA37" s="33"/>
-      <c r="AB37" s="33"/>
+      <c r="T37" s="35"/>
+      <c r="U37" s="35"/>
+      <c r="V37" s="35"/>
+      <c r="W37" s="35"/>
+      <c r="X37" s="35"/>
+      <c r="Y37" s="35"/>
+      <c r="Z37" s="35"/>
+      <c r="AA37" s="35"/>
+      <c r="AB37" s="35"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">

</xml_diff>